<commit_message>
Made Changes--->Excel ,,, CreateEmployeePage(POM))
</commit_message>
<xml_diff>
--- a/testData/Ninza_HRM.xlsx
+++ b/testData/Ninza_HRM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saiap\eclipse-workspace\Assignment2\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B264BDDC-3F2A-4165-B09F-E767C17FED8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BF02F8F-69EA-4146-B548-F4EBED5AA090}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="12240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>ProjectName</t>
   </si>
@@ -109,13 +109,10 @@
     <t>5</t>
   </si>
   <si>
-    <t>VENKAT</t>
-  </si>
-  <si>
     <t>venkat@gmail.com</t>
   </si>
   <si>
-    <t>venkat1223</t>
+    <t>venkat</t>
   </si>
 </sst>
 </file>
@@ -579,17 +576,15 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>27</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>28</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>29</v>
-      </c>
+      <c r="D2" s="3"/>
       <c r="E2" t="s">
         <v>24</v>
       </c>
@@ -600,7 +595,6 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{56837560-10A2-4656-8557-C6EC024ED334}"/>
-    <hyperlink ref="D2" r:id="rId2" display="anvesh@777" xr:uid="{BD0B335B-3133-464C-8E41-717DA1EA7D84}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>